<commit_message>
Revise all portfolio downloads and correct H&R premium threshold
Revise the three PRDs, two investment memos, two presentations, and two financial models for clear professional writing. Preserve requirements, financial assumptions, formulas, scenario outputs, exhibits, and download paths. Reconcile the H&R Block 20% gross IRR threshold to about 16.23% ($58.21/share), and synchronize the existing website correction note.
</commit_message>
<xml_diff>
--- a/HR_Block_PE_LBO_Model.xlsx
+++ b/HR_Block_PE_LBO_Model.xlsx
@@ -333,7 +333,7 @@
   <x:sheetData>
     <x:row r="1" ht="23" customHeight="1">
       <x:c r="A1" s="5" t="str">
-        <x:v>H&amp;R BLOCK | PUBLIC-TO-PRIVATE INVESTMENT CASE</x:v>
+        <x:v>H&amp;R BLOCK TAKE-PRIVATE CASE</x:v>
       </x:c>
       <x:c r="B1" s="5"/>
       <x:c r="C1" s="5"/>
@@ -365,7 +365,7 @@
     </x:row>
     <x:row r="4">
       <x:c r="A4" s="2" t="str">
-        <x:v>AS OF 22 OCTOBER 2026  •  HYPOTHETICAL TRANSACTION  •  USD MILLIONS</x:v>
+        <x:v>AS OF 22 OCTOBER 2026. HYPOTHETICAL TRANSACTION. USD MILLIONS.</x:v>
       </x:c>
       <x:c r="B4" s="2"/>
       <x:c r="C4" s="2"/>
@@ -387,7 +387,7 @@
     </x:row>
     <x:row r="6" ht="23" customHeight="1">
       <x:c r="A6" s="9" t="str">
-        <x:v>UNDERWRITING SNAPSHOT</x:v>
+        <x:v>TRANSACTION SUMMARY</x:v>
       </x:c>
       <x:c r="B6" s="9"/>
       <x:c r="C6" s="9"/>
@@ -534,7 +534,7 @@
     </x:row>
     <x:row r="17" ht="23" customHeight="1">
       <x:c r="A17" s="9" t="str">
-        <x:v>FIVE-YEAR INVESTMENT OUTCOMES</x:v>
+        <x:v>FIVE-YEAR SPONSOR RETURNS</x:v>
       </x:c>
       <x:c r="B17" s="9"/>
       <x:c r="C17" s="9"/>
@@ -743,7 +743,7 @@
     </x:row>
     <x:row r="30">
       <x:c r="A30" s="2" t="str">
-        <x:v>Key rationale: stable cash flow and modest capital intensity, but acquisition premium + borrowing cost impair risk-adjusted returns.</x:v>
+        <x:v>Cash flow and low capital intensity support the case, but the purchase premium and borrowing costs reduce returns.</x:v>
       </x:c>
       <x:c r="B30" s="2"/>
       <x:c r="C30" s="2"/>
@@ -755,7 +755,7 @@
     </x:row>
     <x:row r="31">
       <x:c r="A31" s="2" t="str">
-        <x:v>Key unresolved diligence: seasonal liquidity, tax policy, client retention, automation/AI, senior debt terms, cash accessibility.</x:v>
+        <x:v>Further diligence: seasonal liquidity, tax policy, client retention, AI competition, senior debt terms and available cash.</x:v>
       </x:c>
       <x:c r="B31" s="2"/>
       <x:c r="C31" s="2"/>
@@ -767,7 +767,7 @@
     </x:row>
     <x:row r="32">
       <x:c r="A32" s="2" t="str">
-        <x:v>This is a research case, not a live bid. All forecasts, financing rates, multiples and deal terms are illustrative.</x:v>
+        <x:v>Independent research case. Forecasts, financing rates, multiples and transaction terms are illustrative.</x:v>
       </x:c>
       <x:c r="B32" s="2"/>
       <x:c r="C32" s="2"/>
@@ -803,7 +803,7 @@
   <x:sheetData>
     <x:row r="1" ht="23" customHeight="1">
       <x:c r="A1" s="5" t="str">
-        <x:v>H&amp;R BLOCK | REPORTED FINANCIALS ($ MILLIONS)</x:v>
+        <x:v>H&amp;R BLOCK REPORTED FINANCIALS ($ MILLIONS)</x:v>
       </x:c>
       <x:c r="B1" s="5"/>
       <x:c r="C1" s="5"/>
@@ -1118,7 +1118,7 @@
     </x:row>
     <x:row r="21">
       <x:c r="A21" s="2" t="str">
-        <x:v>FY2025 / FY2026 EBITDA reconciles to the company disclosed non-GAAP EBITDA.</x:v>
+        <x:v>FY2025 and FY2026 EBITDA reconcile to the company's disclosed non-GAAP EBITDA.</x:v>
       </x:c>
       <x:c r="B21" s="2"/>
       <x:c r="C21" s="2"/>
@@ -1130,7 +1130,7 @@
     </x:row>
     <x:row r="22">
       <x:c r="A22" s="2" t="str">
-        <x:v>FY2025 FY2026 financial debt excludes operating leases.</x:v>
+        <x:v>FY2025 and FY2026 financial debt exclude operating leases.</x:v>
       </x:c>
       <x:c r="B22" s="2"/>
       <x:c r="C22" s="2"/>
@@ -1142,7 +1142,7 @@
     </x:row>
     <x:row r="23">
       <x:c r="A23" s="2" t="str">
-        <x:v>Annual cash flow is highly seasonal; June cash is not equivalent to free cash throughout the tax year.</x:v>
+        <x:v>Cash flow is seasonal. June cash does not establish the cash available throughout the tax year.</x:v>
       </x:c>
       <x:c r="B23" s="2"/>
       <x:c r="C23" s="2"/>
@@ -1199,7 +1199,7 @@
   <x:sheetData>
     <x:row r="1" ht="23" customHeight="1">
       <x:c r="A1" s="5" t="str">
-        <x:v>DEAL &amp; SCENARIO INPUTS | BLUE = EDITABLE</x:v>
+        <x:v>TRANSACTION AND SCENARIO INPUTS (BLUE = EDITABLE)</x:v>
       </x:c>
       <x:c r="B1" s="5"/>
       <x:c r="C1" s="5"/>
@@ -1467,7 +1467,7 @@
     </x:row>
     <x:row r="21">
       <x:c r="A21" s="2" t="str">
-        <x:v>Sponsor holding period (years)</x:v>
+        <x:v>Hold period for sensitivity (years)</x:v>
       </x:c>
       <x:c r="B21" s="18" t="n">
         <x:v>5</x:v>
@@ -1575,7 +1575,7 @@
     </x:row>
     <x:row r="29" ht="23" customHeight="1">
       <x:c r="A29" s="9" t="str">
-        <x:v>OPERATING SCENARIOS | ASSUMPTIONS, NOT GUIDANCE</x:v>
+        <x:v>OPERATING SCENARIO ASSUMPTIONS</x:v>
       </x:c>
       <x:c r="B29" s="9"/>
       <x:c r="C29" s="9"/>
@@ -1853,7 +1853,7 @@
     </x:row>
     <x:row r="47">
       <x:c r="A47" s="2" t="str">
-        <x:v>EBITDA vs adjusted EBITDA caveat: FY2027 guidance is adjusted, FY2026 reported historical metric is EBITDA.</x:v>
+        <x:v>FY2027 guidance uses adjusted EBITDA; FY2026 historical results use reported EBITDA. Definitions differ.</x:v>
       </x:c>
       <x:c r="B47" s="2"/>
       <x:c r="C47" s="2"/>
@@ -1865,7 +1865,7 @@
     </x:row>
     <x:row r="48">
       <x:c r="A48" s="2" t="str">
-        <x:v>Lease liabilities, tax assets, stock compensation, seller rollover, and transaction structure require additional diligence.</x:v>
+        <x:v>Further diligence is needed on leases, tax assets, stock compensation, seller rollover and transaction structure.</x:v>
       </x:c>
       <x:c r="B48" s="2"/>
       <x:c r="C48" s="2"/>
@@ -1877,7 +1877,7 @@
     </x:row>
     <x:row r="49">
       <x:c r="A49" s="2" t="str">
-        <x:v>The model assumes full reported cash is transaction-available subject to $500mm sponsor-funded minimum cash; verify foreign/seasonal constraints.</x:v>
+        <x:v>The model uses all reported cash at closing and funds $500mm of opening cash. Foreign and seasonal availability remain unverified.</x:v>
       </x:c>
       <x:c r="B49" s="2"/>
       <x:c r="C49" s="2"/>
@@ -1925,7 +1925,7 @@
   <x:sheetData>
     <x:row r="1" ht="23" customHeight="1">
       <x:c r="A1" s="5" t="str">
-        <x:v>TAKE-PRIVATE | SOURCES &amp; USES ($ MILLIONS)</x:v>
+        <x:v>TAKE-PRIVATE SOURCES AND USES ($ MILLIONS)</x:v>
       </x:c>
       <x:c r="B1" s="5"/>
       <x:c r="C1" s="5"/>
@@ -2505,7 +2505,7 @@
     </x:row>
     <x:row r="43">
       <x:c r="A43" s="2" t="str">
-        <x:v>Assumes debt refinance at book value, available unrestricted cash, no rollover, and no lease-debt capitalization.</x:v>
+        <x:v>Assumes debt refinancing at book value, all reported unrestricted cash available, no seller rollover and no lease-debt capitalization.</x:v>
       </x:c>
       <x:c r="B43" s="2"/>
       <x:c r="C43" s="2"/>
@@ -2517,7 +2517,7 @@
     </x:row>
     <x:row r="44">
       <x:c r="A44" s="2" t="str">
-        <x:v>These assumptions are educational; this is not a financing commitment or executable bid.</x:v>
+        <x:v>Financing rates and terms are illustrative; no lender commitment is assumed.</x:v>
       </x:c>
       <x:c r="B44" s="2"/>
       <x:c r="C44" s="2"/>
@@ -2555,7 +2555,7 @@
   <x:sheetData>
     <x:row r="1" ht="23" customHeight="1">
       <x:c r="A1" s="5" t="str">
-        <x:v>DOWNSIDE CASE | 5-YEAR LBO CASH FLOW AND DEBT SCHEDULE ($ MILLIONS)</x:v>
+        <x:v>DOWNSIDE LBO CASH FLOW AND DEBT ($ MILLIONS)</x:v>
       </x:c>
       <x:c r="B1" s="5"/>
       <x:c r="C1" s="5"/>
@@ -3630,7 +3630,7 @@
     </x:row>
     <x:row r="47">
       <x:c r="A47" s="2" t="str">
-        <x:v>Cash interest on beginning-of-year debt; no revolver, M&amp;A outlays, OID, or tax shield limitation modeled.</x:v>
+        <x:v>Interest uses opening debt balances. No revolver, M&amp;A spending, OID or tax deductibility limit is modeled.</x:v>
       </x:c>
       <x:c r="B47" s="2"/>
       <x:c r="C47" s="2"/>
@@ -3642,7 +3642,7 @@
     </x:row>
     <x:row r="48">
       <x:c r="A48" s="2" t="str">
-        <x:v>All non-mandatory debt paydown applies only to the first-lien term loan; senior notes mature as a bullet at exit.</x:v>
+        <x:v>All discretionary repayments reduce the first-lien term loan. Senior notes remain a bullet payment at exit.</x:v>
       </x:c>
       <x:c r="B48" s="2"/>
       <x:c r="C48" s="2"/>
@@ -3654,7 +3654,7 @@
     </x:row>
     <x:row r="49">
       <x:c r="A49" s="2" t="str">
-        <x:v>Closing cash accumulation may conceal intrayear seasonality / minimum cash needs; confirm with monthly liquidity diligence.</x:v>
+        <x:v>Annual cash balances can miss seasonal funding needs. A monthly liquidity forecast is still needed.</x:v>
       </x:c>
       <x:c r="B49" s="2"/>
       <x:c r="C49" s="2"/>
@@ -3692,7 +3692,7 @@
   <x:sheetData>
     <x:row r="1" ht="23" customHeight="1">
       <x:c r="A1" s="5" t="str">
-        <x:v>BASE CASE | 5-YEAR LBO CASH FLOW AND DEBT SCHEDULE ($ MILLIONS)</x:v>
+        <x:v>BASE LBO CASH FLOW AND DEBT ($ MILLIONS)</x:v>
       </x:c>
       <x:c r="B1" s="5"/>
       <x:c r="C1" s="5"/>
@@ -4767,7 +4767,7 @@
     </x:row>
     <x:row r="47">
       <x:c r="A47" s="2" t="str">
-        <x:v>Cash interest on beginning-of-year debt; no revolver, M&amp;A outlays, OID, or tax shield limitation modeled.</x:v>
+        <x:v>Interest uses opening debt balances. No revolver, M&amp;A spending, OID or tax deductibility limit is modeled.</x:v>
       </x:c>
       <x:c r="B47" s="2"/>
       <x:c r="C47" s="2"/>
@@ -4779,7 +4779,7 @@
     </x:row>
     <x:row r="48">
       <x:c r="A48" s="2" t="str">
-        <x:v>All non-mandatory debt paydown applies only to the first-lien term loan; senior notes mature as a bullet at exit.</x:v>
+        <x:v>All discretionary repayments reduce the first-lien term loan. Senior notes remain a bullet payment at exit.</x:v>
       </x:c>
       <x:c r="B48" s="2"/>
       <x:c r="C48" s="2"/>
@@ -4791,7 +4791,7 @@
     </x:row>
     <x:row r="49">
       <x:c r="A49" s="2" t="str">
-        <x:v>Closing cash accumulation may conceal intrayear seasonality / minimum cash needs; confirm with monthly liquidity diligence.</x:v>
+        <x:v>Annual cash balances can miss seasonal funding needs. A monthly liquidity forecast is still needed.</x:v>
       </x:c>
       <x:c r="B49" s="2"/>
       <x:c r="C49" s="2"/>
@@ -4829,7 +4829,7 @@
   <x:sheetData>
     <x:row r="1" ht="23" customHeight="1">
       <x:c r="A1" s="5" t="str">
-        <x:v>UPSIDE CASE | 5-YEAR LBO CASH FLOW AND DEBT SCHEDULE ($ MILLIONS)</x:v>
+        <x:v>UPSIDE LBO CASH FLOW AND DEBT ($ MILLIONS)</x:v>
       </x:c>
       <x:c r="B1" s="5"/>
       <x:c r="C1" s="5"/>
@@ -5904,7 +5904,7 @@
     </x:row>
     <x:row r="47">
       <x:c r="A47" s="2" t="str">
-        <x:v>Cash interest on beginning-of-year debt; no revolver, M&amp;A outlays, OID, or tax shield limitation modeled.</x:v>
+        <x:v>Interest uses opening debt balances. No revolver, M&amp;A spending, OID or tax deductibility limit is modeled.</x:v>
       </x:c>
       <x:c r="B47" s="2"/>
       <x:c r="C47" s="2"/>
@@ -5916,7 +5916,7 @@
     </x:row>
     <x:row r="48">
       <x:c r="A48" s="2" t="str">
-        <x:v>All non-mandatory debt paydown applies only to the first-lien term loan; senior notes mature as a bullet at exit.</x:v>
+        <x:v>All discretionary repayments reduce the first-lien term loan. Senior notes remain a bullet payment at exit.</x:v>
       </x:c>
       <x:c r="B48" s="2"/>
       <x:c r="C48" s="2"/>
@@ -5928,7 +5928,7 @@
     </x:row>
     <x:row r="49">
       <x:c r="A49" s="2" t="str">
-        <x:v>Closing cash accumulation may conceal intrayear seasonality / minimum cash needs; confirm with monthly liquidity diligence.</x:v>
+        <x:v>Annual cash balances can miss seasonal funding needs. A monthly liquidity forecast is still needed.</x:v>
       </x:c>
       <x:c r="B49" s="2"/>
       <x:c r="C49" s="2"/>
@@ -5966,7 +5966,7 @@
   <x:sheetData>
     <x:row r="1" ht="23" customHeight="1">
       <x:c r="A1" s="5" t="str">
-        <x:v>BASE OPERATIONS | PRICE PREMIUM vs EXIT MULTIPLE</x:v>
+        <x:v>BASE-CASE IRR BY OFFER PREMIUM AND EXIT MULTIPLE</x:v>
       </x:c>
       <x:c r="B1" s="5"/>
       <x:c r="C1" s="5"/>
@@ -6004,7 +6004,7 @@
     </x:row>
     <x:row r="4">
       <x:c r="A4" s="2" t="str">
-        <x:v>Scenario: Base 2031 EBITDA, debt and cash; offer changes sponsor equity and deal fees only.</x:v>
+        <x:v>Base 2031 EBITDA, debt and cash stay fixed. The offer changes sponsor equity and transaction fees only.</x:v>
       </x:c>
       <x:c r="B4" s="2"/>
       <x:c r="C4" s="2"/>
@@ -6327,7 +6327,7 @@
     </x:row>
     <x:row r="16">
       <x:c r="A16" s="2" t="str">
-        <x:v>Sensitivity holds base forecast debt and cash constant across transaction premium changes.</x:v>
+        <x:v>At 7.5x exit, about 16.23% premium ($58.21/share) reaches 20% IRR; exact threshold 16.234532%.</x:v>
       </x:c>
       <x:c r="B16" s="2"/>
       <x:c r="C16" s="2"/>
@@ -6341,7 +6341,7 @@
     </x:row>
     <x:row r="17">
       <x:c r="A17" s="2" t="str">
-        <x:v>Actual capital structure may flex with premium, ratings constraints, and credit-market pricing.</x:v>
+        <x:v>Debt terms may change with premium, ratings or market pricing. At 25% premium and 8.5x exit, IRR is 19.9942%, below 20%.</x:v>
       </x:c>
       <x:c r="B17" s="2"/>
       <x:c r="C17" s="2"/>
@@ -6389,7 +6389,7 @@
   <x:sheetData>
     <x:row r="1" ht="23" customHeight="1">
       <x:c r="A1" s="5" t="str">
-        <x:v>SOURCES, LIMITATIONS AND AUDIT TRAIL</x:v>
+        <x:v>SOURCES AND MODEL LIMITATIONS</x:v>
       </x:c>
       <x:c r="B1" s="5"/>
       <x:c r="C1" s="5"/>
@@ -6588,7 +6588,7 @@
         <x:v>Acquired cash</x:v>
       </x:c>
       <x:c r="B18" s="2" t="str">
-        <x:v>Cash $958.7m at Jun 30 2026 including $238.6m at foreign subsidiaries; not all deployability verified.</x:v>
+        <x:v>$958.7mm cash at June 30, 2026 includes $238.6mm held abroad. Full availability at closing is unverified.</x:v>
       </x:c>
       <x:c r="C18" s="2"/>
       <x:c r="D18" s="2"/>
@@ -6636,7 +6636,7 @@
         <x:v>IRR hurdle / loan rates / offer premium</x:v>
       </x:c>
       <x:c r="B22" s="2" t="str">
-        <x:v>Analyst assumptions; NOT facts about lender terms or board offer.</x:v>
+        <x:v>Analyst assumptions, not lender terms or a board offer.</x:v>
       </x:c>
       <x:c r="C22" s="2"/>
       <x:c r="D22" s="2"/>
@@ -6660,7 +6660,7 @@
         <x:v>Forward model / cash flows</x:v>
       </x:c>
       <x:c r="B24" s="2" t="str">
-        <x:v>Annual simplification, ignores intrayear tax-season revolver, individual debt covenants, OID, and integration costs.</x:v>
+        <x:v>Annual model excludes the seasonal revolver, debt covenants, OID and integration costs.</x:v>
       </x:c>
       <x:c r="C24" s="2"/>
       <x:c r="D24" s="2"/>
@@ -6684,7 +6684,7 @@
         <x:v>Return type</x:v>
       </x:c>
       <x:c r="B26" s="2" t="str">
-        <x:v>Five-year annualized gross sponsor equity IRR before fund fees, carry, financing funding timing.</x:v>
+        <x:v>Gross sponsor equity IRR before fees and carry. Case schedules use five years. B21 changes sensitivity only. Funding timing is simplified.</x:v>
       </x:c>
       <x:c r="C26" s="2"/>
       <x:c r="D26" s="2"/>

</xml_diff>

<commit_message>
Revise all portfolio downloads and correct H&R premium threshold (#3)
Revise the three PRDs, two investment memos, two presentations, and two financial models for clear professional writing. Preserve requirements, financial assumptions, formulas, scenario outputs, exhibits, and download paths. Reconcile the H&R Block 20% gross IRR threshold to about 16.23% ($58.21/share), and synchronize the existing website correction note.
</commit_message>
<xml_diff>
--- a/HR_Block_PE_LBO_Model.xlsx
+++ b/HR_Block_PE_LBO_Model.xlsx
@@ -333,7 +333,7 @@
   <x:sheetData>
     <x:row r="1" ht="23" customHeight="1">
       <x:c r="A1" s="5" t="str">
-        <x:v>H&amp;R BLOCK | PUBLIC-TO-PRIVATE INVESTMENT CASE</x:v>
+        <x:v>H&amp;R BLOCK TAKE-PRIVATE CASE</x:v>
       </x:c>
       <x:c r="B1" s="5"/>
       <x:c r="C1" s="5"/>
@@ -365,7 +365,7 @@
     </x:row>
     <x:row r="4">
       <x:c r="A4" s="2" t="str">
-        <x:v>AS OF 22 OCTOBER 2026  •  HYPOTHETICAL TRANSACTION  •  USD MILLIONS</x:v>
+        <x:v>AS OF 22 OCTOBER 2026. HYPOTHETICAL TRANSACTION. USD MILLIONS.</x:v>
       </x:c>
       <x:c r="B4" s="2"/>
       <x:c r="C4" s="2"/>
@@ -387,7 +387,7 @@
     </x:row>
     <x:row r="6" ht="23" customHeight="1">
       <x:c r="A6" s="9" t="str">
-        <x:v>UNDERWRITING SNAPSHOT</x:v>
+        <x:v>TRANSACTION SUMMARY</x:v>
       </x:c>
       <x:c r="B6" s="9"/>
       <x:c r="C6" s="9"/>
@@ -534,7 +534,7 @@
     </x:row>
     <x:row r="17" ht="23" customHeight="1">
       <x:c r="A17" s="9" t="str">
-        <x:v>FIVE-YEAR INVESTMENT OUTCOMES</x:v>
+        <x:v>FIVE-YEAR SPONSOR RETURNS</x:v>
       </x:c>
       <x:c r="B17" s="9"/>
       <x:c r="C17" s="9"/>
@@ -743,7 +743,7 @@
     </x:row>
     <x:row r="30">
       <x:c r="A30" s="2" t="str">
-        <x:v>Key rationale: stable cash flow and modest capital intensity, but acquisition premium + borrowing cost impair risk-adjusted returns.</x:v>
+        <x:v>Cash flow and low capital intensity support the case, but the purchase premium and borrowing costs reduce returns.</x:v>
       </x:c>
       <x:c r="B30" s="2"/>
       <x:c r="C30" s="2"/>
@@ -755,7 +755,7 @@
     </x:row>
     <x:row r="31">
       <x:c r="A31" s="2" t="str">
-        <x:v>Key unresolved diligence: seasonal liquidity, tax policy, client retention, automation/AI, senior debt terms, cash accessibility.</x:v>
+        <x:v>Further diligence: seasonal liquidity, tax policy, client retention, AI competition, senior debt terms and available cash.</x:v>
       </x:c>
       <x:c r="B31" s="2"/>
       <x:c r="C31" s="2"/>
@@ -767,7 +767,7 @@
     </x:row>
     <x:row r="32">
       <x:c r="A32" s="2" t="str">
-        <x:v>This is a research case, not a live bid. All forecasts, financing rates, multiples and deal terms are illustrative.</x:v>
+        <x:v>Independent research case. Forecasts, financing rates, multiples and transaction terms are illustrative.</x:v>
       </x:c>
       <x:c r="B32" s="2"/>
       <x:c r="C32" s="2"/>
@@ -803,7 +803,7 @@
   <x:sheetData>
     <x:row r="1" ht="23" customHeight="1">
       <x:c r="A1" s="5" t="str">
-        <x:v>H&amp;R BLOCK | REPORTED FINANCIALS ($ MILLIONS)</x:v>
+        <x:v>H&amp;R BLOCK REPORTED FINANCIALS ($ MILLIONS)</x:v>
       </x:c>
       <x:c r="B1" s="5"/>
       <x:c r="C1" s="5"/>
@@ -1118,7 +1118,7 @@
     </x:row>
     <x:row r="21">
       <x:c r="A21" s="2" t="str">
-        <x:v>FY2025 / FY2026 EBITDA reconciles to the company disclosed non-GAAP EBITDA.</x:v>
+        <x:v>FY2025 and FY2026 EBITDA reconcile to the company's disclosed non-GAAP EBITDA.</x:v>
       </x:c>
       <x:c r="B21" s="2"/>
       <x:c r="C21" s="2"/>
@@ -1130,7 +1130,7 @@
     </x:row>
     <x:row r="22">
       <x:c r="A22" s="2" t="str">
-        <x:v>FY2025 FY2026 financial debt excludes operating leases.</x:v>
+        <x:v>FY2025 and FY2026 financial debt exclude operating leases.</x:v>
       </x:c>
       <x:c r="B22" s="2"/>
       <x:c r="C22" s="2"/>
@@ -1142,7 +1142,7 @@
     </x:row>
     <x:row r="23">
       <x:c r="A23" s="2" t="str">
-        <x:v>Annual cash flow is highly seasonal; June cash is not equivalent to free cash throughout the tax year.</x:v>
+        <x:v>Cash flow is seasonal. June cash does not establish the cash available throughout the tax year.</x:v>
       </x:c>
       <x:c r="B23" s="2"/>
       <x:c r="C23" s="2"/>
@@ -1199,7 +1199,7 @@
   <x:sheetData>
     <x:row r="1" ht="23" customHeight="1">
       <x:c r="A1" s="5" t="str">
-        <x:v>DEAL &amp; SCENARIO INPUTS | BLUE = EDITABLE</x:v>
+        <x:v>TRANSACTION AND SCENARIO INPUTS (BLUE = EDITABLE)</x:v>
       </x:c>
       <x:c r="B1" s="5"/>
       <x:c r="C1" s="5"/>
@@ -1467,7 +1467,7 @@
     </x:row>
     <x:row r="21">
       <x:c r="A21" s="2" t="str">
-        <x:v>Sponsor holding period (years)</x:v>
+        <x:v>Hold period for sensitivity (years)</x:v>
       </x:c>
       <x:c r="B21" s="18" t="n">
         <x:v>5</x:v>
@@ -1575,7 +1575,7 @@
     </x:row>
     <x:row r="29" ht="23" customHeight="1">
       <x:c r="A29" s="9" t="str">
-        <x:v>OPERATING SCENARIOS | ASSUMPTIONS, NOT GUIDANCE</x:v>
+        <x:v>OPERATING SCENARIO ASSUMPTIONS</x:v>
       </x:c>
       <x:c r="B29" s="9"/>
       <x:c r="C29" s="9"/>
@@ -1853,7 +1853,7 @@
     </x:row>
     <x:row r="47">
       <x:c r="A47" s="2" t="str">
-        <x:v>EBITDA vs adjusted EBITDA caveat: FY2027 guidance is adjusted, FY2026 reported historical metric is EBITDA.</x:v>
+        <x:v>FY2027 guidance uses adjusted EBITDA; FY2026 historical results use reported EBITDA. Definitions differ.</x:v>
       </x:c>
       <x:c r="B47" s="2"/>
       <x:c r="C47" s="2"/>
@@ -1865,7 +1865,7 @@
     </x:row>
     <x:row r="48">
       <x:c r="A48" s="2" t="str">
-        <x:v>Lease liabilities, tax assets, stock compensation, seller rollover, and transaction structure require additional diligence.</x:v>
+        <x:v>Further diligence is needed on leases, tax assets, stock compensation, seller rollover and transaction structure.</x:v>
       </x:c>
       <x:c r="B48" s="2"/>
       <x:c r="C48" s="2"/>
@@ -1877,7 +1877,7 @@
     </x:row>
     <x:row r="49">
       <x:c r="A49" s="2" t="str">
-        <x:v>The model assumes full reported cash is transaction-available subject to $500mm sponsor-funded minimum cash; verify foreign/seasonal constraints.</x:v>
+        <x:v>The model uses all reported cash at closing and funds $500mm of opening cash. Foreign and seasonal availability remain unverified.</x:v>
       </x:c>
       <x:c r="B49" s="2"/>
       <x:c r="C49" s="2"/>
@@ -1925,7 +1925,7 @@
   <x:sheetData>
     <x:row r="1" ht="23" customHeight="1">
       <x:c r="A1" s="5" t="str">
-        <x:v>TAKE-PRIVATE | SOURCES &amp; USES ($ MILLIONS)</x:v>
+        <x:v>TAKE-PRIVATE SOURCES AND USES ($ MILLIONS)</x:v>
       </x:c>
       <x:c r="B1" s="5"/>
       <x:c r="C1" s="5"/>
@@ -2505,7 +2505,7 @@
     </x:row>
     <x:row r="43">
       <x:c r="A43" s="2" t="str">
-        <x:v>Assumes debt refinance at book value, available unrestricted cash, no rollover, and no lease-debt capitalization.</x:v>
+        <x:v>Assumes debt refinancing at book value, all reported unrestricted cash available, no seller rollover and no lease-debt capitalization.</x:v>
       </x:c>
       <x:c r="B43" s="2"/>
       <x:c r="C43" s="2"/>
@@ -2517,7 +2517,7 @@
     </x:row>
     <x:row r="44">
       <x:c r="A44" s="2" t="str">
-        <x:v>These assumptions are educational; this is not a financing commitment or executable bid.</x:v>
+        <x:v>Financing rates and terms are illustrative; no lender commitment is assumed.</x:v>
       </x:c>
       <x:c r="B44" s="2"/>
       <x:c r="C44" s="2"/>
@@ -2555,7 +2555,7 @@
   <x:sheetData>
     <x:row r="1" ht="23" customHeight="1">
       <x:c r="A1" s="5" t="str">
-        <x:v>DOWNSIDE CASE | 5-YEAR LBO CASH FLOW AND DEBT SCHEDULE ($ MILLIONS)</x:v>
+        <x:v>DOWNSIDE LBO CASH FLOW AND DEBT ($ MILLIONS)</x:v>
       </x:c>
       <x:c r="B1" s="5"/>
       <x:c r="C1" s="5"/>
@@ -3630,7 +3630,7 @@
     </x:row>
     <x:row r="47">
       <x:c r="A47" s="2" t="str">
-        <x:v>Cash interest on beginning-of-year debt; no revolver, M&amp;A outlays, OID, or tax shield limitation modeled.</x:v>
+        <x:v>Interest uses opening debt balances. No revolver, M&amp;A spending, OID or tax deductibility limit is modeled.</x:v>
       </x:c>
       <x:c r="B47" s="2"/>
       <x:c r="C47" s="2"/>
@@ -3642,7 +3642,7 @@
     </x:row>
     <x:row r="48">
       <x:c r="A48" s="2" t="str">
-        <x:v>All non-mandatory debt paydown applies only to the first-lien term loan; senior notes mature as a bullet at exit.</x:v>
+        <x:v>All discretionary repayments reduce the first-lien term loan. Senior notes remain a bullet payment at exit.</x:v>
       </x:c>
       <x:c r="B48" s="2"/>
       <x:c r="C48" s="2"/>
@@ -3654,7 +3654,7 @@
     </x:row>
     <x:row r="49">
       <x:c r="A49" s="2" t="str">
-        <x:v>Closing cash accumulation may conceal intrayear seasonality / minimum cash needs; confirm with monthly liquidity diligence.</x:v>
+        <x:v>Annual cash balances can miss seasonal funding needs. A monthly liquidity forecast is still needed.</x:v>
       </x:c>
       <x:c r="B49" s="2"/>
       <x:c r="C49" s="2"/>
@@ -3692,7 +3692,7 @@
   <x:sheetData>
     <x:row r="1" ht="23" customHeight="1">
       <x:c r="A1" s="5" t="str">
-        <x:v>BASE CASE | 5-YEAR LBO CASH FLOW AND DEBT SCHEDULE ($ MILLIONS)</x:v>
+        <x:v>BASE LBO CASH FLOW AND DEBT ($ MILLIONS)</x:v>
       </x:c>
       <x:c r="B1" s="5"/>
       <x:c r="C1" s="5"/>
@@ -4767,7 +4767,7 @@
     </x:row>
     <x:row r="47">
       <x:c r="A47" s="2" t="str">
-        <x:v>Cash interest on beginning-of-year debt; no revolver, M&amp;A outlays, OID, or tax shield limitation modeled.</x:v>
+        <x:v>Interest uses opening debt balances. No revolver, M&amp;A spending, OID or tax deductibility limit is modeled.</x:v>
       </x:c>
       <x:c r="B47" s="2"/>
       <x:c r="C47" s="2"/>
@@ -4779,7 +4779,7 @@
     </x:row>
     <x:row r="48">
       <x:c r="A48" s="2" t="str">
-        <x:v>All non-mandatory debt paydown applies only to the first-lien term loan; senior notes mature as a bullet at exit.</x:v>
+        <x:v>All discretionary repayments reduce the first-lien term loan. Senior notes remain a bullet payment at exit.</x:v>
       </x:c>
       <x:c r="B48" s="2"/>
       <x:c r="C48" s="2"/>
@@ -4791,7 +4791,7 @@
     </x:row>
     <x:row r="49">
       <x:c r="A49" s="2" t="str">
-        <x:v>Closing cash accumulation may conceal intrayear seasonality / minimum cash needs; confirm with monthly liquidity diligence.</x:v>
+        <x:v>Annual cash balances can miss seasonal funding needs. A monthly liquidity forecast is still needed.</x:v>
       </x:c>
       <x:c r="B49" s="2"/>
       <x:c r="C49" s="2"/>
@@ -4829,7 +4829,7 @@
   <x:sheetData>
     <x:row r="1" ht="23" customHeight="1">
       <x:c r="A1" s="5" t="str">
-        <x:v>UPSIDE CASE | 5-YEAR LBO CASH FLOW AND DEBT SCHEDULE ($ MILLIONS)</x:v>
+        <x:v>UPSIDE LBO CASH FLOW AND DEBT ($ MILLIONS)</x:v>
       </x:c>
       <x:c r="B1" s="5"/>
       <x:c r="C1" s="5"/>
@@ -5904,7 +5904,7 @@
     </x:row>
     <x:row r="47">
       <x:c r="A47" s="2" t="str">
-        <x:v>Cash interest on beginning-of-year debt; no revolver, M&amp;A outlays, OID, or tax shield limitation modeled.</x:v>
+        <x:v>Interest uses opening debt balances. No revolver, M&amp;A spending, OID or tax deductibility limit is modeled.</x:v>
       </x:c>
       <x:c r="B47" s="2"/>
       <x:c r="C47" s="2"/>
@@ -5916,7 +5916,7 @@
     </x:row>
     <x:row r="48">
       <x:c r="A48" s="2" t="str">
-        <x:v>All non-mandatory debt paydown applies only to the first-lien term loan; senior notes mature as a bullet at exit.</x:v>
+        <x:v>All discretionary repayments reduce the first-lien term loan. Senior notes remain a bullet payment at exit.</x:v>
       </x:c>
       <x:c r="B48" s="2"/>
       <x:c r="C48" s="2"/>
@@ -5928,7 +5928,7 @@
     </x:row>
     <x:row r="49">
       <x:c r="A49" s="2" t="str">
-        <x:v>Closing cash accumulation may conceal intrayear seasonality / minimum cash needs; confirm with monthly liquidity diligence.</x:v>
+        <x:v>Annual cash balances can miss seasonal funding needs. A monthly liquidity forecast is still needed.</x:v>
       </x:c>
       <x:c r="B49" s="2"/>
       <x:c r="C49" s="2"/>
@@ -5966,7 +5966,7 @@
   <x:sheetData>
     <x:row r="1" ht="23" customHeight="1">
       <x:c r="A1" s="5" t="str">
-        <x:v>BASE OPERATIONS | PRICE PREMIUM vs EXIT MULTIPLE</x:v>
+        <x:v>BASE-CASE IRR BY OFFER PREMIUM AND EXIT MULTIPLE</x:v>
       </x:c>
       <x:c r="B1" s="5"/>
       <x:c r="C1" s="5"/>
@@ -6004,7 +6004,7 @@
     </x:row>
     <x:row r="4">
       <x:c r="A4" s="2" t="str">
-        <x:v>Scenario: Base 2031 EBITDA, debt and cash; offer changes sponsor equity and deal fees only.</x:v>
+        <x:v>Base 2031 EBITDA, debt and cash stay fixed. The offer changes sponsor equity and transaction fees only.</x:v>
       </x:c>
       <x:c r="B4" s="2"/>
       <x:c r="C4" s="2"/>
@@ -6327,7 +6327,7 @@
     </x:row>
     <x:row r="16">
       <x:c r="A16" s="2" t="str">
-        <x:v>Sensitivity holds base forecast debt and cash constant across transaction premium changes.</x:v>
+        <x:v>At 7.5x exit, about 16.23% premium ($58.21/share) reaches 20% IRR; exact threshold 16.234532%.</x:v>
       </x:c>
       <x:c r="B16" s="2"/>
       <x:c r="C16" s="2"/>
@@ -6341,7 +6341,7 @@
     </x:row>
     <x:row r="17">
       <x:c r="A17" s="2" t="str">
-        <x:v>Actual capital structure may flex with premium, ratings constraints, and credit-market pricing.</x:v>
+        <x:v>Debt terms may change with premium, ratings or market pricing. At 25% premium and 8.5x exit, IRR is 19.9942%, below 20%.</x:v>
       </x:c>
       <x:c r="B17" s="2"/>
       <x:c r="C17" s="2"/>
@@ -6389,7 +6389,7 @@
   <x:sheetData>
     <x:row r="1" ht="23" customHeight="1">
       <x:c r="A1" s="5" t="str">
-        <x:v>SOURCES, LIMITATIONS AND AUDIT TRAIL</x:v>
+        <x:v>SOURCES AND MODEL LIMITATIONS</x:v>
       </x:c>
       <x:c r="B1" s="5"/>
       <x:c r="C1" s="5"/>
@@ -6588,7 +6588,7 @@
         <x:v>Acquired cash</x:v>
       </x:c>
       <x:c r="B18" s="2" t="str">
-        <x:v>Cash $958.7m at Jun 30 2026 including $238.6m at foreign subsidiaries; not all deployability verified.</x:v>
+        <x:v>$958.7mm cash at June 30, 2026 includes $238.6mm held abroad. Full availability at closing is unverified.</x:v>
       </x:c>
       <x:c r="C18" s="2"/>
       <x:c r="D18" s="2"/>
@@ -6636,7 +6636,7 @@
         <x:v>IRR hurdle / loan rates / offer premium</x:v>
       </x:c>
       <x:c r="B22" s="2" t="str">
-        <x:v>Analyst assumptions; NOT facts about lender terms or board offer.</x:v>
+        <x:v>Analyst assumptions, not lender terms or a board offer.</x:v>
       </x:c>
       <x:c r="C22" s="2"/>
       <x:c r="D22" s="2"/>
@@ -6660,7 +6660,7 @@
         <x:v>Forward model / cash flows</x:v>
       </x:c>
       <x:c r="B24" s="2" t="str">
-        <x:v>Annual simplification, ignores intrayear tax-season revolver, individual debt covenants, OID, and integration costs.</x:v>
+        <x:v>Annual model excludes the seasonal revolver, debt covenants, OID and integration costs.</x:v>
       </x:c>
       <x:c r="C24" s="2"/>
       <x:c r="D24" s="2"/>
@@ -6684,7 +6684,7 @@
         <x:v>Return type</x:v>
       </x:c>
       <x:c r="B26" s="2" t="str">
-        <x:v>Five-year annualized gross sponsor equity IRR before fund fees, carry, financing funding timing.</x:v>
+        <x:v>Gross sponsor equity IRR before fees and carry. Case schedules use five years. B21 changes sensitivity only. Funding timing is simplified.</x:v>
       </x:c>
       <x:c r="C26" s="2"/>
       <x:c r="D26" s="2"/>

</xml_diff>